<commit_message>
fix(curtailment): bump _CACHE_VERSION v4->v5 (renames Excel)
Excel unidades_geradoras.xlsx atualizado com 3 renomes na aba
Eólica (EQTL Echo→Equatorial, CGN Brazil→CGN Brasil,
Voltália→Voltalia). _CACHE_VERSION bump força reprocessamento
pra que o df pós-rateio reflita os novos nomes em PROPRIETARIO.
</commit_message>
<xml_diff>
--- a/data/curtailment/unidades_geradoras.xlsx
+++ b/data/curtailment/unidades_geradoras.xlsx
@@ -2731,7 +2731,7 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>EQTL (Echo)</t>
+          <t>Equatorial</t>
         </is>
       </c>
     </row>
@@ -2781,7 +2781,7 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Voltália</t>
+          <t>Voltalia</t>
         </is>
       </c>
     </row>
@@ -2856,7 +2856,7 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>Voltália</t>
+          <t>Voltalia</t>
         </is>
       </c>
     </row>
@@ -2906,7 +2906,7 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>Voltália</t>
+          <t>Voltalia</t>
         </is>
       </c>
     </row>
@@ -2981,7 +2981,7 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>Voltália</t>
+          <t>Voltalia</t>
         </is>
       </c>
     </row>
@@ -4106,7 +4106,7 @@
       </c>
       <c r="E58" t="inlineStr">
         <is>
-          <t>EQTL (Echo)</t>
+          <t>Equatorial</t>
         </is>
       </c>
     </row>
@@ -4131,7 +4131,7 @@
       </c>
       <c r="E59" t="inlineStr">
         <is>
-          <t>EQTL (Echo)</t>
+          <t>Equatorial</t>
         </is>
       </c>
     </row>
@@ -4206,7 +4206,7 @@
       </c>
       <c r="E62" t="inlineStr">
         <is>
-          <t>Voltália</t>
+          <t>Voltalia</t>
         </is>
       </c>
     </row>
@@ -4531,7 +4531,7 @@
       </c>
       <c r="E75" t="inlineStr">
         <is>
-          <t>EQTL (Echo)</t>
+          <t>Equatorial</t>
         </is>
       </c>
     </row>
@@ -4681,7 +4681,7 @@
       </c>
       <c r="E81" t="inlineStr">
         <is>
-          <t>CGN Brazil</t>
+          <t>CGN Brasil</t>
         </is>
       </c>
     </row>
@@ -4831,7 +4831,7 @@
       </c>
       <c r="E87" t="inlineStr">
         <is>
-          <t>CGN Brazil</t>
+          <t>CGN Brasil</t>
         </is>
       </c>
     </row>
@@ -4931,7 +4931,7 @@
       </c>
       <c r="E91" t="inlineStr">
         <is>
-          <t>CGN Brazil</t>
+          <t>CGN Brasil</t>
         </is>
       </c>
     </row>
@@ -5306,7 +5306,7 @@
       </c>
       <c r="E106" t="inlineStr">
         <is>
-          <t>EQTL (Echo)</t>
+          <t>Equatorial</t>
         </is>
       </c>
     </row>
@@ -5656,7 +5656,7 @@
       </c>
       <c r="E120" t="inlineStr">
         <is>
-          <t>CGN Brazil</t>
+          <t>CGN Brasil</t>
         </is>
       </c>
     </row>
@@ -5706,7 +5706,7 @@
       </c>
       <c r="E122" t="inlineStr">
         <is>
-          <t>CGN Brazil</t>
+          <t>CGN Brasil</t>
         </is>
       </c>
     </row>
@@ -5956,7 +5956,7 @@
       </c>
       <c r="E132" t="inlineStr">
         <is>
-          <t>Voltália</t>
+          <t>Voltalia</t>
         </is>
       </c>
     </row>
@@ -6056,7 +6056,7 @@
       </c>
       <c r="E136" t="inlineStr">
         <is>
-          <t>EQTL (Echo)</t>
+          <t>Equatorial</t>
         </is>
       </c>
     </row>
@@ -6756,7 +6756,7 @@
       </c>
       <c r="E164" t="inlineStr">
         <is>
-          <t>EQTL (Echo)</t>
+          <t>Equatorial</t>
         </is>
       </c>
     </row>
@@ -7281,7 +7281,7 @@
       </c>
       <c r="E185" t="inlineStr">
         <is>
-          <t>EQTL (Echo)</t>
+          <t>Equatorial</t>
         </is>
       </c>
     </row>

</xml_diff>